<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-10 Le tapis bleu de Chouchou
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-10.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-10.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le livre rouge de Chouchou</t>
+          <t>Le tapis bleu de Chouchou</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine, coin tapis, puis maison</t>
+          <t>école, coin tapis, puis maison. Couloir savon, chaussons bleus, radiateur, buée</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>La cuillère tape la casserole. Chouchou veut le livre rouge du bateau. Un chuchotement lui serre le ventre. Le soir, il raconte, et papa ouvre le bateau à la maison.</t>
+          <t>Un tic vient du radiateur. Sur un poil, un éclat de tapis brille. Chouchou veut parler maintenant. Elle s'assoit trop vite : l'éclat se cache. Une voix trop près : malaise. Elle ouvre trop vite : les mots se perdent. Elle refuse de foncer, attend, raconte. Merci vécu. Sur le poil, l'éclat de tapis tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La cuillère en bois tape la casserole. Toc. Toc. Ça sent les lentilles chaudes. Une chaussette bleue attend sur la chaise. La vapeur fait un nuage bas. Papa remue tout doucement. Le doudou est dans le sac. Il t'attend ce soir. Je veux le livre rouge. Celui avec le bateau. Il est au coin tapis. Tu écoutes la maîtresse, Chouchou ? Oui, papa. Tu écoutes, puis tu regardes. Oui, maman. En ce moment, Chouchou s'assoit. Le tapis est bleu, tout doux. Ça chatouille un peu les genoux. Un rayon touche une page. Les livres sentent le papier. Les chaussons sont en rang. On écoute. Ensuite, on range les livres. Chouchou aime écouter. Il cherche le livre rouge. Le dos du livre est rêche. Il l'ouvre. Le bateau a une voile. La voile est grande, maîtresse. Oui, Chouchou. Tu as bien écouté. On range, maintenant. Chouchou pose le livre dans le bac. Les pages font un petit bruit. Plus tard, quelqu'un parle tout bas. Chouchou entend parler d'un secret. Son ventre se serre. Il pose les mains sur le tapis. Je raconterai à la maison. Le soir, papa coupe des carottes. Ça sent la terre. Les ronds orange brillent. Tu as faim, Chouchou ? Chouchou vient près de la table. Il a encore le ventre serré. Le doudou attend dans le sac.</t>
+          <t>Un tic vient du radiateur. La vitre est tiède, un peu floue. Une buée ronde tient sur le verre. Le savon du couloir pique le nez. Tes chaussons bleus sont près du banc. Ils sont froids, papa. Enfile-les, un pied puis l'autre. Le chausson gauche colle un peu. Il colle, maman. Tire vers toi. Le pied droit entre, plus facile. On va au coin tapis ? Oui, tout de suite ! Chouchou marche dans le couloir. Les chaussons bleus font un petit choc. Le tapis bleu attend au fond. Les poils sont courts, un peu rèches. Sur un poil, un éclat de tapis brille. Il brille, papa ! C'est le bleu, sous la lumière. Je m'assois, maintenant ! Pendant que je pose les sacs ? Oui, tout de suite ! En ce moment, Chouchou s'assoit. Elle pose le genou trop vite. L'éclat se cache sous le genou. Il est parti ! Le sourire de Chouchou disparaît. Dans sa poitrine, ça tape fort. L'envie et l'inquiétude se bousculent. Tu le cherches, Chouchou ? Oui, papa. Papa se baisse à sa hauteur. Elle lève le genou, lente. L'éclat de tapis tremble, puis tient. Il est là. On dit bonjour ? Oui. La maîtresse parle près des chaises. Bonjour les enfants. Bonjour, maîtresse. Chouchou pose les genoux sur le bleu. Ça chatouille un peu les genoux. Un camarade s'approche près du tapis. Il parle près de l'oreille. Chouchou sent un malaise dans le ventre. Son ventre se serre, tout petit. Je veux le dire, maintenant. Elle ouvre la bouche, trop vite. Les mots se perdent dans la classe. Personne n'entend le malaise. Chouchou referme la bouche, un instant. Le nœud reste dans le ventre. Le soir, la porte s'ouvre. Ça sent le savon de la maison. Le radiateur fait tic, près de la vitre. Une buée mince tient sur le verre. Te voilà, Chouchou. Tes chaussons bleus sont mouillés ? Un peu, papa. Viens près de la table. Chouchou pose les chaussons près du radiateur. Le ventre est serré, tout petit. Elle regarde papa, près de la table. Elle ouvre la bouche, un peu.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Hadrien est à l'école. C'est le coin tapis. La maîtresse parle. Hadrien aime &lt;emphasis level="moderate"&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on range les livres. Hadrien range un livre. Il écoute bien. Plus tard, un camarade chuchote. Il dit : c'est un secret. Ne le dis pas à la maison. Hadrien sent un malaise. Son ventre est serré. Le soir, papa coupe des carottes. Ça sent la terre. Hadrien vient raconter à la maison. Il dit : papa, j'ai eu un malaise. Un camarade a parlé d'un secret. Maman l'écoute aussi. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un tic vient du radiateur. La vitre est tiède, un peu floue. Une buée ronde tient sur le verre. Le savon du couloir pique le nez. Tes chaussons bleus sont près du banc. Ils sont froids, papa. Enfile-les, un pied puis l'autre. Le chausson gauche colle un peu. Il colle, maman. Tire vers toi. Le pied droit entre, plus facile. On va au coin tapis ? Oui, tout de suite ! Chouchou marche dans le couloir. Les chaussons bleus font un petit choc. Le tapis bleu attend au fond. Les poils sont courts, un peu rèches. Sur un poil, un &lt;emphasis level="moderate"&gt;éclat de tapis&lt;/emphasis&gt; brille. Il brille, papa ! C'est le bleu, sous la lumière. Je m'assois, maintenant ! Pendant que je pose les sacs ? Oui, tout de suite ! En ce moment, Chouchou s'assoit. Elle pose le genou trop vite. L'éclat se cache sous le genou. Il est parti ! Le sourire de Chouchou disparaît. Dans sa poitrine, ça tape fort. L'envie et l'inquiétude se bousculent. Tu le cherches, Chouchou ? Oui, papa. Papa se baisse à sa hauteur. Elle lève le genou, lente. L'éclat de tapis tremble, puis tient. Il est là. On dit bonjour ? Oui. La maîtresse parle près des chaises. Bonjour les enfants. Bonjour, maîtresse. Chouchou pose les genoux sur le bleu. Ça chatouille un peu les genoux. Un camarade s'approche près du tapis. Il parle près de l'oreille. Chouchou sent un malaise dans le ventre. Son ventre se serre, tout petit. Je veux le dire, maintenant. Elle ouvre la bouche, trop vite. Les mots se perdent dans la classe. Personne n'entend le malaise. Chouchou referme la bouche, un instant. Le nœud reste dans le ventre. Le soir, la porte s'ouvre. Ça sent le savon de la maison. Le radiateur fait tic, près de la vitre. Une buée mince tient sur le verre. Te voilà, Chouchou. Tes chaussons bleus sont mouillés ? Un peu, papa. Viens près de la table. Chouchou pose les chaussons près du radiateur. Le ventre est serré, tout petit. Elle regarde papa, près de la table. Elle ouvre la bouche, un peu.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Hadrien est à l'école. C'est le coin tapis. La maîtresse parle. Hadrien aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on range les livres. Hadrien range un livre. Il écoute bien. Plus tard, un camarade chuchote. Il dit : c'est un secret. Ne le dis pas à la maison. Hadrien sent un malaise. Son ventre est serré. Le soir, papa coupe des carottes. Ça sent la terre. Hadrien vient raconter à la maison. Il dit : papa, j'ai eu un malaise. Un camarade a parlé d'un secret. Maman l'écoute aussi. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman.&lt;/slow&gt; [pause]</t>
+          <t>Un tic vient du radiateur. La vitre est tiède, un peu floue. Une buée ronde tient sur le verre. Le savon du couloir pique le nez. Tes chaussons bleus sont près du banc. Ils sont froids, papa. Enfile-les, un pied puis l'autre. Le chausson gauche colle un peu. Il colle, maman. Tire vers toi. Le pied droit entre, plus facile. On va au coin tapis ? Oui, tout de suite ! Chouchou marche dans le couloir. Les chaussons bleus font un petit choc. Le tapis bleu attend au fond. Les poils sont courts, un peu rèches. Sur un poil, un &lt;emphasis&gt;éclat de tapis&lt;/emphasis&gt; brille. Il brille, papa ! C'est le bleu, sous la lumière. Je m'assois, maintenant ! Pendant que je pose les sacs ? Oui, tout de suite ! En ce moment, Chouchou s'assoit. Elle pose le genou trop vite. L'éclat se cache sous le genou. Il est parti ! Le sourire de Chouchou disparaît. Dans sa poitrine, ça tape fort. L'envie et l'inquiétude se bousculent. Tu le cherches, Chouchou ? Oui, papa. Papa se baisse à sa hauteur. Elle lève le genou, lente. L'éclat de tapis tremble, puis tient. Il est là. On dit bonjour ? Oui. La maîtresse parle près des chaises. Bonjour les enfants. Bonjour, maîtresse. Chouchou pose les genoux sur le bleu. Ça chatouille un peu les genoux. Un camarade s'approche près du tapis. Il parle près de l'oreille. Chouchou sent un malaise dans le ventre. Son ventre se serre, tout petit. Je veux le dire, maintenant. Elle ouvre la bouche, trop vite. Les mots se perdent dans la classe. Personne n'entend le malaise. Chouchou referme la bouche, un instant. Le nœud reste dans le ventre. Le soir, la porte s'ouvre. Ça sent le savon de la maison. Le radiateur fait tic, près de la vitre. Une buée mince tient sur le verre. Te voilà, Chouchou. Tes chaussons bleus sont mouillés ? Un peu, papa. Viens près de la table. Chouchou pose les chaussons près du radiateur. Le ventre est serré, tout petit. Elle regarde papa, près de la table. Elle ouvre la bouche, un peu. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de tapis</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,63 +1324,85 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis malaise; intensite=2; destinataire=enfant; sous_texte=elle_veut_parler_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La cuillère en bois tape la casserole.
-narrateur|Toc.
-narrateur|Toc.
-narrateur|Ça sent les lentilles chaudes.
-narrateur|Une chaussette bleue attend sur la chaise.
-narrateur|La vapeur fait un nuage bas.
-narrateur|Papa remue tout doucement.
-maman|Le doudou est dans le sac.
-maman|Il t'attend ce soir.
-enfant-m|Je veux le livre rouge.
-enfant-m|Celui avec le bateau.
-papa|Il est au coin tapis.
-papa|Tu écoutes la maîtresse, Chouchou ?
-enfant-m|Oui, papa.
-maman|Tu écoutes, puis tu regardes.
-enfant-m|Oui, maman.
+          <t>narrateur|Un tic vient du radiateur.
+narrateur|La vitre est tiède, un peu floue.
+narrateur|Une buée ronde tient sur le verre.
+narrateur|Le savon du couloir pique le nez.
+papa|Tes chaussons bleus sont près du banc.
+enfant-f|Ils sont froids, papa.
+maman|Enfile-les, un pied puis l'autre.
+narrateur|Le chausson gauche colle un peu.
+enfant-f|Il colle, maman.
+maman|Tire vers toi.
+narrateur|Le pied droit entre, plus facile.
+papa|On va au coin tapis ?
+enfant-f|Oui, tout de suite !
+narrateur|Chouchou marche dans le couloir.
+narrateur|Les chaussons bleus font un petit choc.
+narrateur|Le tapis bleu attend au fond.
+narrateur|Les poils sont courts, un peu rèches.
+narrateur|Sur un poil, un éclat de tapis brille.
+enfant-f|Il brille, papa !
+papa|C'est le bleu, sous la lumière.
+enfant-f|Je m'assois, maintenant !
+maman|Pendant que je pose les sacs ?
+enfant-f|Oui, tout de suite !
 narrateur|En ce moment, Chouchou s'assoit.
-narrateur|Le tapis est bleu, tout doux.
+narrateur|Elle pose le genou trop vite.
+narrateur|L'éclat se cache sous le genou.
+enfant-f|Il est parti !
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, ça tape fort.
+narrateur|L'envie et l'inquiétude se bousculent.
+papa|Tu le cherches, Chouchou ?
+enfant-f|Oui, papa.
+narrateur|Papa se baisse à sa hauteur.
+narrateur|Elle lève le genou, lente.
+narrateur|L'éclat de tapis tremble, puis tient.
+enfant-f|Il est là.
+papa|On dit bonjour ?
+enfant-f|Oui.
+narrateur|La maîtresse parle près des chaises.
+maitresse|Bonjour les enfants.
+enfant-f|Bonjour, maîtresse.
+narrateur|Chouchou pose les genoux sur le bleu.
 narrateur|Ça chatouille un peu les genoux.
-narrateur|Un rayon touche une page.
-narrateur|Les livres sentent le papier.
-narrateur|Les chaussons sont en rang.
-maitresse|On écoute.
-maitresse|Ensuite, on range les livres.
-narrateur|Chouchou aime écouter.
-narrateur|Il cherche le livre rouge.
-narrateur|Le dos du livre est rêche.
-narrateur|Il l'ouvre.
-narrateur|Le bateau a une voile.
-enfant-m|La voile est grande, maîtresse.
-maitresse|Oui, Chouchou.
-maitresse|Tu as bien écouté.
-maitresse|On range, maintenant.
-narrateur|Chouchou pose le livre dans le bac.
-narrateur|Les pages font un petit bruit.
-narrateur|Plus tard, quelqu'un parle tout bas.
-narrateur|Chouchou entend parler d'un secret.
-narrateur|Son ventre se serre.
-narrateur|Il pose les mains sur le tapis.
-enfant-m|Je raconterai à la maison.
-narrateur|Le soir, papa coupe des carottes.
-narrateur|Ça sent la terre.
-narrateur|Les ronds orange brillent.
-papa|Tu as faim, Chouchou ?
-narrateur|Chouchou vient près de la table.
-narrateur|Il a encore le ventre serré.
-narrateur|Le doudou attend dans le sac.</t>
+narrateur|Un camarade s'approche près du tapis.
+narrateur|Il parle près de l'oreille.
+narrateur|Chouchou sent un malaise dans le ventre.
+narrateur|Son ventre se serre, tout petit.
+enfant-f|Je veux le dire, maintenant.
+narrateur|Elle ouvre la bouche, trop vite.
+narrateur|Les mots se perdent dans la classe.
+narrateur|Personne n'entend le malaise.
+narrateur|Chouchou referme la bouche, un instant.
+narrateur|Le nœud reste dans le ventre.
+narrateur|Le soir, la porte s'ouvre.
+narrateur|Ça sent le savon de la maison.
+narrateur|Le radiateur fait tic, près de la vitre.
+narrateur|Une buée mince tient sur le verre.
+papa|Te voilà, Chouchou.
+papa|Tes chaussons bleus sont mouillés ?
+enfant-f|Un peu, papa.
+maman|Viens près de la table.
+narrateur|Chouchou pose les chaussons près du radiateur.
+narrateur|Le ventre est serré, tout petit.
+narrateur|Elle regarde papa, près de la table.
+narrateur|Elle ouvre la bouche, un peu.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>casserole,pages</t>
+          <t>radiateur,chaussons</t>
         </is>
       </c>
     </row>
@@ -1407,17 +1429,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a un malaise. Que fait-il ?</t>
+          <t>Chouchou a un malaise. Que fait-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Hadrien a un malaise. Que fait-il ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Chouchou a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Hadrien a un malaise. Que fait-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Chouchou a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1427,7 +1449,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>raconter | il raconte | à papa | à la maison | écouter</t>
+          <t>raconter | elle raconte | à papa | à la maison | écouter | elle attend | attendre | son tour | malaise</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1442,7 +1464,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il raconte à papa. Que fait Chouchou ?</t>
+          <t>Elle raconte à papa. Que fait Chouchou ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1480,7 +1502,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1488,10 +1510,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1506,34 +1528,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1542,13 +1568,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1558,13 +1584,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_raconte_quand_on_l_entend; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Chouchou a un malaise.
-narrateur|Que fait-il ?</t>
+narrateur|Que fait-elle ?</t>
         </is>
       </c>
     </row>
@@ -1591,17 +1617,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Papa, j'ai eu un malaise. Quelqu'un a parlé d'un secret. Maman s'approche. Tu as bien fait de raconter. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter. À papa ou à maman. Chouchou respire. J'ai vu le bateau. Dans le livre rouge. On a un livre, ici aussi. Tu veux le voir ? Oui. Papa prend un livre sur l'étagère. La couverture est un peu usée. Il y a un bateau, lui aussi.</t>
+          <t>Chouchou ouvre la bouche trop vite. Papa, l'oreille, le nœud, le tapis ! Papa n'a pas fini sa phrase. Les chaussons sèchent, Chouchou. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Chouchou refuse de foncer sur les mots. Elle referme la bouche, un instant. Elle pose les mains à plat. Elle écoute la maison, un instant. Le radiateur fait tic, près de toi. Papa pose sa tasse sur la table. La buée tient sur la vitre. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Sur le poil, l'éclat de tapis brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé près de mon oreille. Ça a serré, ici. Chouchou montre son ventre, tout petit. Merci, Chouchou. Papa a entendu toute la phrase. Tu as faim, un peu ? Un peu, maman. Le ventre de Chouchou se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Hadrien a écouté la maîtresse. Il a raconté son malaise à la maison. Papa et maman sont là.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou ouvre la bouche trop vite. Papa, l'oreille, le nœud, le tapis ! Papa n'a pas fini sa phrase. Les chaussons sèchent, Chouchou. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Chouchou refuse de foncer sur les mots. Elle referme la bouche, un instant. Elle pose les mains à plat. Elle écoute la maison, un instant. Le radiateur fait tic, près de toi. Papa pose sa tasse sur la table. La buée tient sur la vitre. Maman n'a pas fini non plus. Chouchou attend que le &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive. Sur le poil, l'éclat de tapis brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé près de mon oreille. Ça a serré, ici. Chouchou montre son ventre, tout petit. Merci, Chouchou. Papa a entendu toute la phrase. Tu as faim, un peu ? Un peu, maman. Le ventre de Chouchou se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Hadrien a écouté la maîtresse. Il a raconté son malaise à la maison. Papa et maman sont là.&lt;/slow&gt; [pause]</t>
+          <t>Chouchou ouvre la bouche trop vite. Papa, l'oreille, le nœud, le tapis ! Papa n'a pas fini sa phrase. Les chaussons sèchent, Chouchou. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Chouchou refuse de foncer sur les mots. Elle referme la bouche, un instant. Elle pose les mains à plat. Elle écoute la maison, un instant. Le radiateur fait tic, près de toi. Papa pose sa tasse sur la table. La buée tient sur la vitre. Maman n'a pas fini non plus. Chouchou attend que le &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive. Sur le poil, l'éclat de tapis brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé près de mon oreille. Ça a serré, ici. Chouchou montre son ventre, tout petit. Merci, Chouchou. Papa a entendu toute la phrase. Tu as faim, un peu ? Un peu, maman. Le ventre de Chouchou se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1648,18 +1674,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1680,28 +1706,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>silence</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1710,10 +1740,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1722,31 +1752,48 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Papa, j'ai eu un malaise.
-enfant-m|Quelqu'un a parlé d'un secret.
-narrateur|Maman s'approche.
-maman|Tu as bien fait de raconter.
-maman|On aime écouter la maîtresse.
-papa|Si tu as un malaise, tu viens raconter.
-papa|À papa ou à maman.
-narrateur|Chouchou respire.
-enfant-m|J'ai vu le bateau.
-enfant-m|Dans le livre rouge.
-maman|On a un livre, ici aussi.
-maman|Tu veux le voir ?
-enfant-m|Oui.
-narrateur|Papa prend un livre sur l'étagère.
-narrateur|La couverture est un peu usée.
-narrateur|Il y a un bateau, lui aussi.</t>
+          <t>narrateur|Chouchou ouvre la bouche trop vite.
+enfant-f|Papa, l'oreille, le nœud, le tapis !
+narrateur|Papa n'a pas fini sa phrase.
+papa|Les chaussons sèchent, Chouchou.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Chouchou refuse de foncer sur les mots.
+narrateur|Elle referme la bouche, un instant.
+narrateur|Elle pose les mains à plat.
+narrateur|Elle écoute la maison, un instant.
+papa|Le radiateur fait tic, près de toi.
+narrateur|Papa pose sa tasse sur la table.
+maman|La buée tient sur la vitre.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Chouchou attend que le silence arrive.
+narrateur|Sur le poil, l'éclat de tapis brille.
+enfant-f|Il est là.
+enfant-f|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-f|Un camarade a parlé près de mon oreille.
+enfant-f|Ça a serré, ici.
+narrateur|Chouchou montre son ventre, tout petit.
+papa|Merci, Chouchou.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu as faim, un peu ?
+enfant-f|Un peu, maman.
+narrateur|Le ventre de Chouchou se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>tasse,table</t>
         </is>
       </c>
     </row>
@@ -1773,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa ouvre le livre. La voile est un peu pliée. Il va jusqu'à demain. Je te tiens la main ? Oui, papa. Sa main est chaude. Tu prends le doudou ? Oui, maman. Le doudou sent la maison. Papa verse un verre d'eau. Chouchou boit une gorgée. L'eau est fraîche. La cuillère repose dans la casserole.</t>
+          <t>Tu t'assois, près du tapis ? Oui, le bleu. Un petit tapis bleu attend près du radiateur. Chouchou veut s'asseoir tout de suite. Elle pose le genou trop vite. Le tapis glisse un peu. Oh. Elle veut tout dire d'un coup. L'école, l'oreille, le bleu ! Les mots se bousculent dans sa bouche. Personne n'entend la fin. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute le radiateur, un instant. Elle lève le genou, lente. Un poil brille, pâle, sous le genou. Comme à l'école, papa. Tu le vois, toi ? Oui, sur le bleu. Elle s'assoit, sans presser. On entend presque le couloir. Le savon, et les chaussons. Tu restes un peu ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Hadrien boit un verre d'eau. Papa lui tient la &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tu t'assois, près du tapis ? Oui, le bleu. Un petit tapis bleu attend près du radiateur. Chouchou veut s'asseoir tout de suite. Elle pose le &lt;emphasis level="moderate"&gt;genou&lt;/emphasis&gt; trop vite. Le tapis glisse un peu. Oh. Elle veut tout dire d'un coup. L'école, l'oreille, le bleu ! Les mots se bousculent dans sa bouche. Personne n'entend la fin. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute le radiateur, un instant. Elle lève le genou, lente. Un poil brille, pâle, sous le genou. Comme à l'école, papa. Tu le vois, toi ? Oui, sur le bleu. Elle s'assoit, sans presser. On entend presque le couloir. Le savon, et les chaussons. Tu restes un peu ? Oui, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Hadrien boit un verre d'eau. Papa lui tient la &lt;emphasis&gt;main&lt;/emphasis&gt;.&lt;/slow&gt; [pause]</t>
+          <t>Tu t'assois, près du tapis ? Oui, le bleu. Un petit tapis bleu attend près du radiateur. Chouchou veut s'asseoir tout de suite. Elle pose le &lt;emphasis&gt;genou&lt;/emphasis&gt; trop vite. Le tapis glisse un peu. Oh. Elle veut tout dire d'un coup. L'école, l'oreille, le bleu ! Les mots se bousculent dans sa bouche. Personne n'entend la fin. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute le radiateur, un instant. Elle lève le genou, lente. Un poil brille, pâle, sous le genou. Comme à l'école, papa. Tu le vois, toi ? Oui, sur le bleu. Elle s'assoit, sans presser. On entend presque le couloir. Le savon, et les chaussons. Tu restes un peu ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1830,18 +1877,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1864,30 +1911,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>genou</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1896,10 +1943,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1908,29 +1955,45 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sur_le_tapis; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa ouvre le livre.
-narrateur|La voile est un peu pliée.
-enfant-m|Il va jusqu'à demain.
-papa|Je te tiens la main ?
-enfant-m|Oui, papa.
-narrateur|Sa main est chaude.
-maman|Tu prends le doudou ?
-enfant-m|Oui, maman.
-narrateur|Le doudou sent la maison.
-narrateur|Papa verse un verre d'eau.
-narrateur|Chouchou boit une gorgée.
-maman|L'eau est fraîche.
-narrateur|La cuillère repose dans la casserole.</t>
+          <t>papa|Tu t'assois, près du tapis ?
+enfant-f|Oui, le bleu.
+narrateur|Un petit tapis bleu attend près du radiateur.
+narrateur|Chouchou veut s'asseoir tout de suite.
+narrateur|Elle pose le genou trop vite.
+narrateur|Le tapis glisse un peu.
+enfant-f|Oh.
+narrateur|Elle veut tout dire d'un coup.
+enfant-f|L'école, l'oreille, le bleu !
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Personne n'entend la fin.
+enfant-f|Oh.
+narrateur|Chouchou refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle écoute le radiateur, un instant.
+narrateur|Elle lève le genou, lente.
+narrateur|Un poil brille, pâle, sous le genou.
+enfant-f|Comme à l'école, papa.
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur le bleu.
+narrateur|Elle s'assoit, sans presser.
+maman|On entend presque le couloir.
+enfant-f|Le savon, et les chaussons.
+papa|Tu restes un peu ?
+enfant-f|Oui, papa.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>verre,pages</t>
+          <t>tapis,radiateur</t>
         </is>
       </c>
     </row>
@@ -1957,17 +2020,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai vu le bateau. J'ai écouté. Puis j'ai raconté. On t'a écouté. Bravo, Chouchou.</t>
+          <t>Les chaussons sèchent près du radiateur. Le petit tapis bleu reste au sol. Comme au coin tapis, maman. Tu le vois, toi ? Oui, sur un poil. On est bien, ici. La buée tient, mince, sur la vitre. Chouchou glisse la main, sans se presser. On l'entend, papa. Tu l'entends sur le bleu ? Oui, le tic. Le savon reste dans l'air. L'éclat de tapis tient sur le poil.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai vu le bateau. J'ai écouté. Puis j'ai raconté. On t'a écouté. Bravo, Chouchou.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les chaussons sèchent près du radiateur. Le petit tapis bleu reste au sol. Comme au coin tapis, maman. Tu le vois, toi ? Oui, sur un poil. On est bien, ici. La buée tient, mince, sur la vitre. Chouchou glisse la main, sans se presser. On l'entend, papa. Tu l'entends sur le bleu ? Oui, le tic. Le savon reste dans l'air. L'&lt;emphasis level="moderate"&gt;éclat de tapis&lt;/emphasis&gt; tient sur le poil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les chaussons sèchent près du radiateur. Le petit tapis bleu reste au sol. Comme au coin tapis, maman. Tu le vois, toi ? Oui, sur un poil. On est bien, ici. La buée tient, mince, sur la vitre. Chouchou glisse la main, sans se presser. On l'entend, papa. Tu l'entends sur le bleu ? Oui, le tic. Le savon reste dans l'air. L'&lt;emphasis&gt;éclat de tapis&lt;/emphasis&gt; tient sur le poil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2014,7 +2077,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2022,10 +2085,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2034,12 +2097,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2048,17 +2111,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tapis</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2067,11 +2134,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2080,28 +2147,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_poil; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai vu le bateau.
-enfant-m|J'ai écouté.
-enfant-m|Puis j'ai raconté.
-maman|On t'a écouté.
-papa|Bravo, Chouchou.</t>
+          <t>narrateur|Les chaussons sèchent près du radiateur.
+narrateur|Le petit tapis bleu reste au sol.
+enfant-f|Comme au coin tapis, maman.
+maman|Tu le vois, toi ?
+enfant-f|Oui, sur un poil.
+papa|On est bien, ici.
+narrateur|La buée tient, mince, sur la vitre.
+narrateur|Chouchou glisse la main, sans se presser.
+enfant-f|On l'entend, papa.
+papa|Tu l'entends sur le bleu ?
+enfant-f|Oui, le tic.
+narrateur|Le savon reste dans l'air.
+narrateur|L'éclat de tapis tient sur le poil.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>radiateur,vitre</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2179,6 +2263,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>